<commit_message>
Ship workout dose rules, site content admin, and VPS deploy while dropping unused trainer and calculator code.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/seeds/foods_catalog_perfect_v1.xlsx
+++ b/seeds/foods_catalog_perfect_v1.xlsx
@@ -5413,7 +5413,7 @@
       </c>
       <c r="C49" s="29" t="inlineStr">
         <is>
-          <t>Cải xoăn Kale</t>
+          <t>Cải xoăn</t>
         </is>
       </c>
       <c r="D49" s="29" t="inlineStr"/>
@@ -19555,7 +19555,7 @@
       </c>
       <c r="C207" s="29" t="inlineStr">
         <is>
-          <t>Cánh gà khúc giữa (Mid-joint wing)</t>
+          <t>Cánh gà khúc giữa</t>
         </is>
       </c>
       <c r="D207" s="29" t="inlineStr"/>
@@ -28302,7 +28302,7 @@
       </c>
       <c r="C304" s="29" t="inlineStr">
         <is>
-          <t>Cá hồi Atlantic (sống)</t>
+          <t>Cá hồi Đại Tây Dương</t>
         </is>
       </c>
       <c r="D304" s="29" t="inlineStr">
@@ -28480,7 +28480,7 @@
       </c>
       <c r="C306" s="29" t="inlineStr">
         <is>
-          <t>Cá hồi sockeye</t>
+          <t>Cá hồi đỏ</t>
         </is>
       </c>
       <c r="D306" s="29" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="C325" s="23" t="inlineStr">
         <is>
-          <t>Cá tra / basa phi lê</t>
+          <t>Cá tra / cá basa phi lê</t>
         </is>
       </c>
       <c r="D325" s="23" t="inlineStr"/>

</xml_diff>